<commit_message>
Add Now Playing paywall for Timer/Clock, move AirPlay to floating action bar, and Phase 6 features
- Gate Sleep Timer and Sleep Clock behind premium paywall in NowPlayingView
- Move AirPlay button from top bar to floating action bar center (free for all users)
- Fix floating action bar layout with fixed-width buttons to prevent overflow
- Add analytics tracking, live activities, now playing manager, and sound files
- Update onboarding, shortcuts, and various UI views with design polish

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Asset-Tracker.xlsx
+++ b/Asset-Tracker.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,8 +56,11 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <color rgb="00006100"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +75,17 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001A1D2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -101,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -117,6 +131,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3932,7 +3954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4181,131 +4203,139 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Heavy Rain</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>~500 KB</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Pixabay (juliush)</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>414 KB</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>Must be seamless loop</t>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>26s loop, processed via ffmpeg, loudnorm -14 LUFS</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Light Rain</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>~500 KB</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Pixabay (DRAGON-STUDIO)</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>560 KB</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr"/>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>45s loop, Calming Rain Loop, processed via ffmpeg</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Rain on Tent</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>~500 KB</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Pixabay (nils_vega)</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>744 KB</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr"/>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>45s loop → rain_on_roof.m4a, processed via ffmpeg</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -4349,45 +4379,49 @@
       <c r="I10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Thunderstorm</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>~600 KB</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Pixabay (calystheranylen)</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>796 KB</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr"/>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>50s loop, rain+thunder, fade in/out 3s</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -4595,217 +4629,239 @@
       <c r="I16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Birds Singing</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Nature</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>~500 KB</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Pixabay (freesound_community)</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>715 KB</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr"/>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>45s loop → birds.m4a, ffmpeg loudnorm -14 LUFS</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Crickets</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Nature</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>~400 KB</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Pixabay (freesound_community)</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>714 KB</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr"/>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>45s loop → crickets.m4a, ffmpeg loudnorm -14 LUFS</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Nature</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>~400 KB</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Pixabay (DRAGON-STUDIO)</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>432 KB</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I19" s="3" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>27s loop → wind.m4a (source 30s), ffmpeg loudnorm</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Forest Ambience</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Nature</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>~500 KB</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Pixabay (audiopapkin)</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>719 KB</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>45s loop → forest.m4a, ffmpeg loudnorm -14 LUFS</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Campfire</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Fire</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>20b</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Rustling Leaves</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>~400 KB</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr"/>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Pixabay (freesound_community)</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>510 KB</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>32s loop → leaves.m4a, ffmpeg loudnorm -14 LUFS</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Fireplace</t>
+          <t>Campfire</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -4842,405 +4898,411 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Fireplace</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Freesound.org / Pixabay</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>~400 KB</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Fan</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>Machine</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t>Freesound.org / Record yourself</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>~400 KB</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G24" s="9" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>Easy to self-record</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="n">
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>Processed via ffmpeg → fan.m4a (mono)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Air Conditioner</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>Machine</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>Freesound.org / Record yourself</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>~400 KB</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>Easy to self-record</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="n">
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>Processed via ffmpeg → ac.m4a (mono)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Clothes Dryer</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>Machine</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>Freesound.org / Record yourself</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>~400 KB</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>Easy to self-record</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Airplane Interior</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>Processed via ffmpeg → dryer.m4a (mono)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Washing Machine</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>Machine</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>~500 KB</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I26" s="3" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Train</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Urban</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>~500 KB</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr"/>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>Pixabay</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>freesound_community-washing-machine-71102</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>256 KB</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="inlineStr">
+        <is>
+          <t>Processed via ffmpeg → washing_machine.m4a (mono, 16s)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Airplane Interior</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Machine</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Freesound.org / Pixabay</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>~500 KB</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Train</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Freesound.org / Pixabay</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>~500 KB</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t>Processed via ffmpeg → train.m4a</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>City Streets</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>Urban</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>Freesound.org / Pixabay</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>~500 KB</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G30" s="9" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Cat Purring</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Nature</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>~400 KB</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Wind Chimes (Bamboo)</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Nature</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>~400 KB</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>Processed via ffmpeg → city_traffic.m4a</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Cafe Ambience</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Pixabay</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>freesound_community-ambience-coffee-shop-5-17059</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>716 KB</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Tibetan Singing Bowl</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>Freesound.org / Pixabay</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>~500 KB</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>Premium</t>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="inlineStr">
+        <is>
+          <t>Processed via ffmpeg → cafe.m4a (45s)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Underwater Bubbles</t>
+          <t>Cat Purring</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -5260,7 +5322,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -5268,24 +5330,20 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
+      <c r="I32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Japanese Garden</t>
+          <t>Wind Chimes (Bamboo)</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -5300,7 +5358,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>~500 KB</t>
+          <t>~400 KB</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -5321,11 +5379,11 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Northern Lights Drone</t>
+          <t>Tibetan Singing Bowl</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -5366,16 +5424,16 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Cabin in the Rain</t>
+          <t>Underwater Bubbles</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Rain</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -5390,7 +5448,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>~500 KB</t>
+          <t>~400 KB</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -5411,16 +5469,16 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Midnight Forest</t>
+          <t>Japanese Garden</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -5456,16 +5514,16 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Desert Wind</t>
+          <t>Northern Lights Drone</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -5480,7 +5538,7 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>~400 KB</t>
+          <t>~500 KB</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -5501,16 +5559,16 @@
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Snow Falling</t>
+          <t>Cabin in the Rain</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Rain</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -5525,7 +5583,7 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>~400 KB</t>
+          <t>~500 KB</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -5546,16 +5604,16 @@
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Coffee Shop</t>
+          <t>Midnight Forest</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -5591,16 +5649,16 @@
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Library Ambience</t>
+          <t>Desert Wind</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -5636,51 +5694,187 @@
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Snow Falling</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Freesound.org / Pixabay</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>~400 KB</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Coffee Shop</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Freesound.org / Pixabay</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>~500 KB</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Library Ambience</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Freesound.org / Pixabay</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>~400 KB</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Vinyl Crackle</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E44" s="3" t="inlineStr">
         <is>
           <t>Freesound.org / Pixabay</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F44" s="3" t="inlineStr">
         <is>
           <t>~300 KB</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G44" s="3" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I41" s="3" t="inlineStr">
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="1" t="inlineStr">
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
         <is>
           <t>SOUND SOURCES: Freesound.org (CC) | Pixabay Audio (free commercial) | Zapsplat.com | Record yourself (fan, dryer, AC)</t>
         </is>

</xml_diff>